<commit_message>
modif detail excel mesure
</commit_message>
<xml_diff>
--- a/source/Catalogue_mesures_Power_BI_v2.xlsx
+++ b/source/Catalogue_mesures_Power_BI_v2.xlsx
@@ -8,33 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bialx-my.sharepoint.com/personal/manuel_ramanitra_bial-r_com/Documents/Documents/Manu Projet/01_PBI_Gestion_Projet/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="11_B23E7286C988CDFB4DD72739E97E2063EF3EE654" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C7D796C-690F-44F1-A103-D22DCE9D8AC5}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="11_B23E7286C988CDFB4DD72739E97E2063EF3EE654" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{273D982B-340B-44BA-AAC0-A774E17C728A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil2" sheetId="5" r:id="rId1"/>
-    <sheet name="Catalogue des mesures" sheetId="1" r:id="rId2"/>
-    <sheet name="Synthèse" sheetId="2" r:id="rId3"/>
-    <sheet name="Notes" sheetId="3" r:id="rId4"/>
+    <sheet name="Catalogue des mesures" sheetId="1" r:id="rId1"/>
+    <sheet name="Synthèse" sheetId="2" r:id="rId2"/>
+    <sheet name="Notes" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogue des mesures'!$A$1:$G$71</definedName>
-    <definedName name="_xlcn.WorksheetConnection_CataloguedesmesuresGG1" hidden="1">'Catalogue des mesures'!$G:$G</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalogue des mesures'!$A$1:$G$71</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <pivotCaches>
-    <pivotCache cacheId="14" r:id="rId5"/>
-  </pivotCaches>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{FCE2AD5D-F65C-4FA6-A056-5C36A1767C68}">
-      <x15:dataModel>
-        <x15:modelTables>
-          <x15:modelTable id="Plage" name="Plage" connection="WorksheetConnection_Catalogue des mesures!$G:$G"/>
-        </x15:modelTables>
-      </x15:dataModel>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -50,31 +37,8 @@
 </workbook>
 </file>
 
-<file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
-<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
-  <connection id="1" xr16:uid="{8ED3CDC7-F4A3-4CCA-A7FE-5CDBAC06404E}" keepAlive="1" name="ThisWorkbookDataModel" description="Modèle de données" type="5" refreshedVersion="8" minRefreshableVersion="5" background="1">
-    <dbPr connection="Data Model Connection" command="Model" commandType="1"/>
-    <olapPr sendLocale="1" rowDrillCount="1000"/>
-    <extLst>
-      <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
-        <x15:connection id="" model="1"/>
-      </ext>
-    </extLst>
-  </connection>
-  <connection id="2" xr16:uid="{BD046736-4C2B-439E-A1C1-D08527AE3724}" name="WorksheetConnection_Catalogue des mesures!$G:$G" type="102" refreshedVersion="8" minRefreshableVersion="5">
-    <extLst>
-      <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{DE250136-89BD-433C-8126-D09CA5730AF9}">
-        <x15:connection id="Plage" autoDelete="1">
-          <x15:rangePr sourceName="_xlcn.WorksheetConnection_CataloguedesmesuresGG1"/>
-        </x15:connection>
-      </ext>
-    </extLst>
-  </connection>
-</connections>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="270">
   <si>
     <t>Nom de la mesure</t>
   </si>
@@ -1150,15 +1114,6 @@
   </si>
   <si>
     <t>La colonne Expression DAX inclut désormais la déclaration MEASURE 'Nom de la mesure' = suivie de l'expression originale. Les commentaires DAX // et -- ont été conservés à partir du fichier source.</t>
-  </si>
-  <si>
-    <t>Étiquettes de lignes</t>
-  </si>
-  <si>
-    <t>(vide)</t>
-  </si>
-  <si>
-    <t>Total général</t>
   </si>
 </sst>
 </file>
@@ -1262,7 +1217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1292,10 +1247,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1311,159 +1262,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Manuel RAMANITRA" refreshedDate="46318.709474074072" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{3656AD96-200A-4E32-9B1F-60C9F7431C26}">
-  <cacheSource type="external" connectionId="1"/>
-  <cacheFields count="1">
-    <cacheField name="[Plage].[Catégorie de la mesure].[Catégorie de la mesure]" caption="Catégorie de la mesure" numFmtId="0" level="1">
-      <sharedItems containsBlank="1" count="13">
-        <m/>
-        <s v="Budget &amp; coûts"/>
-        <s v="Décisions"/>
-        <s v="Délais &amp; avancement"/>
-        <s v="Gestion des changements"/>
-        <s v="Incidents"/>
-        <s v="Livrables"/>
-        <s v="Pilotage général"/>
-        <s v="Qualité"/>
-        <s v="Reporting"/>
-        <s v="Risques"/>
-        <s v="Synthèse &amp; statut"/>
-        <s v="Tâches &amp; ressources"/>
-      </sharedItems>
-    </cacheField>
-  </cacheFields>
-  <cacheHierarchies count="3">
-    <cacheHierarchy uniqueName="[Plage].[Catégorie de la mesure]" caption="Catégorie de la mesure" attribute="1" defaultMemberUniqueName="[Plage].[Catégorie de la mesure].[All]" allUniqueName="[Plage].[Catégorie de la mesure].[All]" dimensionUniqueName="[Plage]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="0"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Plage]" caption="__XL_Count Plage" measure="1" displayFolder="" measureGroup="Plage" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <dimensions count="2">
-    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
-    <dimension name="Plage" uniqueName="[Plage]" caption="Plage"/>
-  </dimensions>
-  <measureGroups count="1">
-    <measureGroup name="Plage" caption="Plage"/>
-  </measureGroups>
-  <maps count="1">
-    <map measureGroup="0" dimension="1"/>
-  </maps>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-    <ext xmlns:xlpdsc="http://schemas.microsoft.com/office/spreadsheetml/2026/pivotDataSourceClean" uri="{F4336242-56EE-4DD3-A5F7-E900642BF6E9}">
-      <xlpdsc:dataSourceClean>1</xlpdsc:dataSourceClean>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B4EE36EE-C4A1-4496-8D00-129CDD78EF9C}" name="Tableau croisé dynamique2" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:A17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="1">
-    <pivotField axis="axisRow" allDrilled="1" showAll="0" dataSourceSort="1" defaultAttributeDrillState="1">
-      <items count="14">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="14">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <pivotHierarchies count="3">
-    <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-  </pivotHierarchies>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <rowHierarchiesUsage count="1">
-    <rowHierarchyUsage hierarchyUsage="0"/>
-  </rowHierarchiesUsage>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{E67621CE-5B39-4880-91FE-76760E9C1902}">
-      <x15:pivotTableUISettings sourceDataName="WorksheetConnection_Catalogue des mesures!$G:$G">
-        <x15:activeTabTopLevelEntity name="[Plage]"/>
-      </x15:pivotTableUISettings>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1750,94 +1548,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{157A4B57-347C-49BA-86B5-E94A46357E4C}">
-  <dimension ref="A3:A17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="22.26953125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" s="14" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" s="14" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" s="14" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" s="14" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" s="14" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" s="14" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A10" s="14" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A11" s="14" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A13" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A14" s="14" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A15" s="14" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A16" s="14" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" s="14" t="s">
-        <v>272</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3490,7 +3200,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3627,7 +3337,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>